<commit_message>
docs: set weekly plan start to 6 July 2026 in timeline and week 1 report
</commit_message>
<xml_diff>
--- a/reports/09-timeline/Project_Timeline.xlsx
+++ b/reports/09-timeline/Project_Timeline.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">Project start (Monday of week 1)</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumed. Change this date and every week updates.</t>
+    <t xml:space="preserve">Plan start date. Change it and every week updates.</t>
   </si>
   <si>
     <t xml:space="preserve">Week</t>
@@ -483,24 +483,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -532,11 +536,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -795,351 +799,351 @@
   <dimension ref="A1:H20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="70"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="n">
-        <v>46300</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" s="4" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="n">
+    <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="8" t="n">
         <f aca="false">$B$3+7*(A6-1)</f>
-        <v>46300</v>
-      </c>
-      <c r="C6" s="7" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C6" s="8" t="n">
         <f aca="false">B6+6</f>
-        <v>46306</v>
-      </c>
-      <c r="D6" s="6" t="s">
+        <v>46215</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="n">
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <f aca="false">$B$3+7*(A7-1)</f>
-        <v>46307</v>
-      </c>
-      <c r="C7" s="10" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C7" s="11" t="n">
         <f aca="false">B7+6</f>
-        <v>46313</v>
-      </c>
-      <c r="D7" s="9" t="s">
+        <v>46222</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="n">
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="8" t="n">
         <f aca="false">$B$3+7*(A8-1)</f>
-        <v>46314</v>
-      </c>
-      <c r="C8" s="7" t="n">
+        <v>46223</v>
+      </c>
+      <c r="C8" s="8" t="n">
         <f aca="false">B8+6</f>
-        <v>46320</v>
-      </c>
-      <c r="D8" s="6" t="s">
+        <v>46229</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="H8" s="6"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="n">
+      <c r="H8" s="7"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="11" t="n">
         <f aca="false">$B$3+7*(A9-1)</f>
-        <v>46321</v>
-      </c>
-      <c r="C9" s="10" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C9" s="11" t="n">
         <f aca="false">B9+6</f>
-        <v>46327</v>
-      </c>
-      <c r="D9" s="9" t="s">
+        <v>46236</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="H9" s="9"/>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="n">
+      <c r="H9" s="10"/>
+    </row>
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="8" t="n">
         <f aca="false">$B$3+7*(A10-1)</f>
-        <v>46328</v>
-      </c>
-      <c r="C10" s="7" t="n">
+        <v>46237</v>
+      </c>
+      <c r="C10" s="8" t="n">
         <f aca="false">B10+6</f>
-        <v>46334</v>
-      </c>
-      <c r="D10" s="6" t="s">
+        <v>46243</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="H10" s="6"/>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="n">
+      <c r="H10" s="7"/>
+    </row>
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="11" t="n">
         <f aca="false">$B$3+7*(A11-1)</f>
-        <v>46335</v>
-      </c>
-      <c r="C11" s="10" t="n">
+        <v>46244</v>
+      </c>
+      <c r="C11" s="11" t="n">
         <f aca="false">B11+6</f>
-        <v>46341</v>
-      </c>
-      <c r="D11" s="9" t="s">
+        <v>46250</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="H11" s="9"/>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="n">
+      <c r="H11" s="10"/>
+    </row>
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="8" t="n">
         <f aca="false">$B$3+7*(A12-1)</f>
-        <v>46342</v>
-      </c>
-      <c r="C12" s="7" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C12" s="8" t="n">
         <f aca="false">B12+6</f>
-        <v>46348</v>
-      </c>
-      <c r="D12" s="6" t="s">
+        <v>46257</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="H12" s="7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="n">
+    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="11" t="n">
         <f aca="false">$B$3+7*(A13-1)</f>
-        <v>46349</v>
-      </c>
-      <c r="C13" s="10" t="n">
+        <v>46258</v>
+      </c>
+      <c r="C13" s="11" t="n">
         <f aca="false">B13+6</f>
-        <v>46355</v>
-      </c>
-      <c r="D13" s="9" t="s">
+        <v>46264</v>
+      </c>
+      <c r="D13" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="G13" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="H13" s="9"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="n">
+      <c r="H13" s="10"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="8" t="n">
         <f aca="false">$B$3+7*(A14-1)</f>
-        <v>46356</v>
-      </c>
-      <c r="C14" s="7" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C14" s="8" t="n">
         <f aca="false">B14+6</f>
-        <v>46362</v>
-      </c>
-      <c r="D14" s="6" t="s">
+        <v>46271</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G14" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="H14" s="6"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="n">
+      <c r="H14" s="7"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="11" t="n">
         <f aca="false">$B$3+7*(A15-1)</f>
-        <v>46363</v>
-      </c>
-      <c r="C15" s="10" t="n">
+        <v>46272</v>
+      </c>
+      <c r="C15" s="11" t="n">
         <f aca="false">B15+6</f>
-        <v>46369</v>
-      </c>
-      <c r="D15" s="9" t="s">
+        <v>46278</v>
+      </c>
+      <c r="D15" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="H15" s="9"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="H15" s="10"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="12" t="n">
+      <c r="B18" s="13" t="n">
         <f aca="false">COUNTIF(G6:G15,"Done")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="13" t="n">
         <f aca="false">COUNTIF(G6:G15,"In progress")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="12" t="n">
+      <c r="B20" s="13" t="n">
         <f aca="false">COUNTIF(G6:G15,"Planned")</f>
         <v>8</v>
       </c>
@@ -1169,342 +1173,342 @@
   <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="22"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="n">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="6" t="n">
+      <c r="D4" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="10" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="10" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="n">
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="10" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="10" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="10" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="2" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="12" t="n">
+      <c r="C19" s="13" t="n">
         <f aca="false">COUNTIF(F4:F17,"Done*")</f>
         <v>9</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="2" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="12" t="n">
+      <c r="C20" s="13" t="n">
         <f aca="false">COUNTIF(F4:F17,"Made, not committed")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="2" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="12" t="n">
+      <c r="C21" s="13" t="n">
         <f aca="false">COUNTIF(F4:F17,"In progress")</f>
         <v>2</v>
       </c>
@@ -1528,162 +1532,162 @@
   <dimension ref="A1:D15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="6" t="n">
+      <c r="B4" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D10" s="6"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="D10" s="7"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D11" s="6"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="D11" s="7"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="13" t="n">
         <f aca="false">SUM(B4:B11)</f>
         <v>100</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="13" t="n">
         <f aca="false">SUMIF(C4:C11,"&lt;&gt;Not started",B4:B11)</f>
         <v>70</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="B15" s="13" t="n">
+      <c r="B15" s="14" t="n">
         <f aca="false">B14/B13</f>
         <v>0.7</v>
       </c>

</xml_diff>

<commit_message>
docs: refresh commit log, week 1 report and timeline after author fix
</commit_message>
<xml_diff>
--- a/reports/09-timeline/Project_Timeline.xlsx
+++ b/reports/09-timeline/Project_Timeline.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="110">
   <si>
     <t xml:space="preserve">POS System: 10-week project timeline</t>
   </si>
@@ -69,7 +69,7 @@
     <t xml:space="preserve">Done</t>
   </si>
   <si>
-    <t xml:space="preserve">e154036, 2016d55, 76f7ec5, ae83e2e, b4a6f5a, 6891d41 to 5e1ae71 (12 Redux commits), ba6b43c, ba99aad, c61014c</t>
+    <t xml:space="preserve">13dc390, 4584088, 80c721c, ef6144e, dbcae3a, 7ab1196 to 9809d35 (11 Redux commits), 046f470, 67e0b4c, 9e2ca1a, 8172cb7, 11645a2, b0ebffe</t>
   </si>
   <si>
     <t xml:space="preserve">Design and SRS</t>
@@ -84,7 +84,7 @@
     <t xml:space="preserve">In progress</t>
   </si>
   <si>
-    <t xml:space="preserve">Diagrams made, commit pending. Customers.jsx added by a teammate. Redux part 2 assigned to Subhash.</t>
+    <t xml:space="preserve">Diagrams committed (11645a2). Branch Manager, Cashier and Onboarding pages in progress by teammates. SRS and Redux part 2 pending.</t>
   </si>
   <si>
     <t xml:space="preserve">Frontend: auth and super admin</t>
@@ -171,19 +171,19 @@
     <t xml:space="preserve">Evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Team repo created and report folders set up</t>
+    <t xml:space="preserve">Team repo and report folders set up</t>
   </si>
   <si>
     <t xml:space="preserve">Weekly Progress</t>
   </si>
   <si>
-    <t xml:space="preserve">ae83e2e, 0de054b</t>
+    <t xml:space="preserve">80c721c, 4584088</t>
   </si>
   <si>
     <t xml:space="preserve">Full Spring Boot backend uploaded</t>
   </si>
   <si>
-    <t xml:space="preserve">76f7ec5</t>
+    <t xml:space="preserve">ef6144e</t>
   </si>
   <si>
     <t xml:space="preserve">Project idea, abstract and objectives</t>
@@ -192,7 +192,7 @@
     <t xml:space="preserve">Idea &amp; Abstract</t>
   </si>
   <si>
-    <t xml:space="preserve">e154036</t>
+    <t xml:space="preserve">see commit_log.csv</t>
   </si>
   <si>
     <t xml:space="preserve">Features, modules and tech stack</t>
@@ -201,31 +201,64 @@
     <t xml:space="preserve">SRS / Documentation</t>
   </si>
   <si>
-    <t xml:space="preserve">2016d55</t>
+    <t xml:space="preserve">13dc390</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend folder structure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ddf392b, 751e82d (subhash8729)</t>
   </si>
   <si>
     <t xml:space="preserve">Frontend config, API client and utils</t>
   </si>
   <si>
-    <t xml:space="preserve">b4a6f5a</t>
+    <t xml:space="preserve">dbcae3a</t>
   </si>
   <si>
     <t xml:space="preserve">Redux Toolkit part 1: adminDashboard, auth, branch, branchAnalytics, cart, category, customer, employee, inventory, onboarding, order</t>
   </si>
   <si>
-    <t xml:space="preserve">6891d41, fa37aff, b800862, 59c7e45, 3742915, 391ed0a, c59138e, ded8c80, 7fd0937, ce4e04a, 5e1ae71</t>
+    <t xml:space="preserve">7ab1196, 0abb5fc, 06b282a, 09a4708, 26e7b01, 8d7cd95, b04b449, ed775da, e426064, c579b5a, 9809d35</t>
   </si>
   <si>
     <t xml:space="preserve">Commit log updated</t>
   </si>
   <si>
-    <t xml:space="preserve">ba6b43c</t>
+    <t xml:space="preserve">046f470, 67e0b4c, 8360f7e</t>
   </si>
   <si>
     <t xml:space="preserve">Postman testing report (2 parts)</t>
   </si>
   <si>
-    <t xml:space="preserve">ba99aad, c61014c</t>
+    <t xml:space="preserve">9e2ca1a, 8172cb7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UML, ER and architecture diagrams (20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11645a2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">README with weekly plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b0ebffe, cdd3a24, b4bee2d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-week timeline and marks tracker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">75398a4, 28069ac, 65daf38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Week 1 report and weekly template</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4430a3c, 7ce4830</t>
   </si>
   <si>
     <t xml:space="preserve">API test case sheet (96 cases)</t>
@@ -237,40 +270,31 @@
     <t xml:space="preserve">Made, not committed</t>
   </si>
   <si>
-    <t xml:space="preserve">UML, ER and architecture diagrams (20)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POS_UML_Diagrams_v2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">README updated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">README.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branch Manager Customers page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Teammate commit, see git log</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Done by teammate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cashier pages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Teammate, not pushed yet</t>
+    <t xml:space="preserve">Branch Manager pages: customers, dashboard, cashier performance (choubisavishvas-web)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3197520, bb95311, db9c60b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cashier pages: sidebar, cart, components (iamvkb7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3d1187e, deff443, 655d718, 2d48633, 7974ef5, 7faddd4, 76a311a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onboarding owner details page (tanyasingh077)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7307504</t>
   </si>
   <si>
     <t xml:space="preserve">Redux Toolkit part 2 and globleState.js</t>
   </si>
   <si>
-    <t xml:space="preserve">Subhash, not pushed yet</t>
+    <t xml:space="preserve">Not pushed yet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pending</t>
   </si>
   <si>
     <t xml:space="preserve">Progress by marks component</t>
@@ -297,16 +321,16 @@
     <t xml:space="preserve">Design (Use-case, Class, ER)</t>
   </si>
   <si>
+    <t xml:space="preserve">20 diagrams committed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly Progress (tracking sheet)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Started</t>
   </si>
   <si>
-    <t xml:space="preserve">Diagrams made, commit pending.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weekly Progress (tracking sheet)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commit log and this timeline. Update every week.</t>
+    <t xml:space="preserve">Commit log, timeline and weekly reports. Update every week.</t>
   </si>
   <si>
     <t xml:space="preserve">Backend and Redux part 1 done, pages in progress.</t>
@@ -483,28 +507,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -536,11 +556,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -799,351 +819,351 @@
   <dimension ref="A1:H20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="70"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="n">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="n">
         <v>46209</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="8" t="n">
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="n">
         <f aca="false">$B$3+7*(A6-1)</f>
         <v>46209</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="7" t="n">
         <f aca="false">B6+6</f>
         <v>46215</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="n">
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="10" t="n">
         <f aca="false">$B$3+7*(A7-1)</f>
         <v>46216</v>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="10" t="n">
         <f aca="false">B7+6</f>
         <v>46222</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="12" t="s">
+      <c r="G7" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="7" t="n">
         <f aca="false">$B$3+7*(A8-1)</f>
         <v>46223</v>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="7" t="n">
         <f aca="false">B8+6</f>
         <v>46229</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H8" s="7"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="n">
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="10" t="n">
         <f aca="false">$B$3+7*(A9-1)</f>
         <v>46230</v>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C9" s="10" t="n">
         <f aca="false">B9+6</f>
         <v>46236</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="12" t="s">
+      <c r="G9" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="H9" s="10"/>
-    </row>
-    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="n">
+      <c r="H9" s="9"/>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="7" t="n">
         <f aca="false">$B$3+7*(A10-1)</f>
         <v>46237</v>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="7" t="n">
         <f aca="false">B10+6</f>
         <v>46243</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="n">
+      <c r="H10" s="6"/>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="10" t="n">
         <f aca="false">$B$3+7*(A11-1)</f>
         <v>46244</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="10" t="n">
         <f aca="false">B11+6</f>
         <v>46250</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="G11" s="12" t="s">
+      <c r="G11" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="H11" s="10"/>
-    </row>
-    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="n">
+      <c r="H11" s="9"/>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="7" t="n">
         <f aca="false">$B$3+7*(A12-1)</f>
         <v>46251</v>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="7" t="n">
         <f aca="false">B12+6</f>
         <v>46257</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="n">
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="10" t="n">
         <f aca="false">$B$3+7*(A13-1)</f>
         <v>46258</v>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="10" t="n">
         <f aca="false">B13+6</f>
         <v>46264</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="G13" s="12" t="s">
+      <c r="G13" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="H13" s="10"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="n">
+      <c r="H13" s="9"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="7" t="n">
         <f aca="false">$B$3+7*(A14-1)</f>
         <v>46265</v>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="7" t="n">
         <f aca="false">B14+6</f>
         <v>46271</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H14" s="7"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="n">
+      <c r="H14" s="6"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="11" t="n">
+      <c r="B15" s="10" t="n">
         <f aca="false">$B$3+7*(A15-1)</f>
         <v>46272</v>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="10" t="n">
         <f aca="false">B15+6</f>
         <v>46278</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="G15" s="12" t="s">
+      <c r="G15" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="H15" s="10"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+      <c r="H15" s="9"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="13" t="n">
+      <c r="B18" s="12" t="n">
         <f aca="false">COUNTIF(G6:G15,"Done")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="13" t="n">
+      <c r="B19" s="12" t="n">
         <f aca="false">COUNTIF(G6:G15,"In progress")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="13" t="n">
+      <c r="B20" s="12" t="n">
         <f aca="false">COUNTIF(G6:G15,"Planned")</f>
         <v>8</v>
       </c>
@@ -1170,347 +1190,427 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="7" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="7" t="s">
+      <c r="D4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="10" t="s">
+      <c r="D5" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="D6" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="7" t="s">
+      <c r="D6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="D7" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="10" t="s">
+      <c r="D7" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="7" t="s">
+      <c r="D8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="10" t="s">
+      <c r="D9" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="n">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D10" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="F10" s="7" t="s">
+      <c r="D11" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="C11" s="10" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="F11" s="10" t="s">
+      <c r="D12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="C12" s="7" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="D13" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="C14" s="7" t="s">
+      <c r="D17" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="D18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="n">
+      <c r="D19" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" s="12" t="n">
+        <f aca="false">COUNTIF(F4:F21,"Done*")</f>
         <v>13</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="F16" s="7" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C24" s="12" t="n">
+        <f aca="false">COUNTIF(F4:F21,"Made, not committed")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="n">
-        <v>14</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D17" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C19" s="13" t="n">
-        <f aca="false">COUNTIF(F4:F17,"Done*")</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C20" s="13" t="n">
-        <f aca="false">COUNTIF(F4:F17,"Made, not committed")</f>
+      <c r="C25" s="12" t="n">
+        <f aca="false">COUNTIF(F4:F21,"In progress")</f>
         <v>3</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="13" t="n">
-        <f aca="false">COUNTIF(F4:F17,"In progress")</f>
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1532,162 +1632,162 @@
   <dimension ref="A1:D15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="C3" s="6" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="D3" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="7" t="n">
+      <c r="B4" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+      <c r="D4" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="C5" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B6" s="7" t="n">
+      <c r="C5" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B6" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="C6" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="B7" s="7" t="n">
+      <c r="C6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="C7" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="C8" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+      <c r="C8" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="D9" s="7" t="s">
+      <c r="C9" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="B10" s="7" t="n">
+      <c r="D10" s="6"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B11" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D10" s="7"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B11" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D11" s="7"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="B13" s="13" t="n">
+      <c r="C11" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="D11" s="6"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B13" s="12" t="n">
         <f aca="false">SUM(B4:B11)</f>
         <v>100</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="B14" s="13" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B14" s="12" t="n">
         <f aca="false">SUMIF(C4:C11,"&lt;&gt;Not started",B4:B11)</f>
         <v>70</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B15" s="14" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B15" s="13" t="n">
         <f aca="false">B14/B13</f>
         <v>0.7</v>
       </c>

</xml_diff>